<commit_message>
Shape Menu around tap-to-plan cooking with a merged buy list and paired fridge leftovers.
Keep matching sides visible, skip freezer-pack protein at shop, group chicken prep and cookbook wings, and put the book tab last.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/prep-labels.xlsx
+++ b/public/prep-labels.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="85">
   <si>
     <t>id</t>
   </si>
@@ -31,7 +31,7 @@
     <t>Годен до</t>
   </si>
   <si>
-    <t>beef-strips-pepper</t>
+    <t>beef-strips-stroganoff</t>
   </si>
   <si>
     <t>Говядина</t>
@@ -43,18 +43,12 @@
     <t>600 г</t>
   </si>
   <si>
-    <t>Говядина с перцем в соевом</t>
+    <t>Бефстроганов</t>
   </si>
   <si>
     <t>до 03.12.2026</t>
   </si>
   <si>
-    <t>beef-strips-stroganoff</t>
-  </si>
-  <si>
-    <t>Бефстроганов</t>
-  </si>
-  <si>
     <t>beef-cubes-goulash-w2</t>
   </si>
   <si>
@@ -67,30 +61,27 @@
     <t>beef-cubes-potato</t>
   </si>
   <si>
+    <t>Картофель тушёный с говядиной</t>
+  </si>
+  <si>
+    <t>beef-large-pulled</t>
+  </si>
+  <si>
+    <t>крупный кусок</t>
+  </si>
+  <si>
+    <t>450 г</t>
+  </si>
+  <si>
+    <t>Рваная говядина в красном вине</t>
+  </si>
+  <si>
+    <t>beef-large-roast</t>
+  </si>
+  <si>
     <t>700 г</t>
   </si>
   <si>
-    <t>Картофель тушёный с мясом</t>
-  </si>
-  <si>
-    <t>beef-cubes-goulash-w4</t>
-  </si>
-  <si>
-    <t>beef-large-pulled</t>
-  </si>
-  <si>
-    <t>крупный кусок</t>
-  </si>
-  <si>
-    <t>450 г</t>
-  </si>
-  <si>
-    <t>Рваная говядина в красном вине</t>
-  </si>
-  <si>
-    <t>beef-large-roast</t>
-  </si>
-  <si>
     <t>Говядина в горчично-травной корочке</t>
   </si>
   <si>
@@ -100,10 +91,16 @@
     <t>фарш</t>
   </si>
   <si>
+    <t>Паста болоньезе</t>
+  </si>
+  <si>
+    <t>beef-mince-navy</t>
+  </si>
+  <si>
     <t>500 г</t>
   </si>
   <si>
-    <t>Болоньезе</t>
+    <t>Макароны по-флотски</t>
   </si>
   <si>
     <t>beef-meatballs-pack</t>
@@ -124,13 +121,13 @@
     <t>до 03.11.2026</t>
   </si>
   <si>
-    <t>chick-cubes-pasta-mushroom</t>
+    <t>chick-cubes-pasta-zucchini</t>
   </si>
   <si>
     <t>550 г</t>
   </si>
   <si>
-    <t>Паста с курицей и грибами</t>
+    <t>Паста с курицей и кабачком</t>
   </si>
   <si>
     <t>chick-strips-stroganoff</t>
@@ -157,7 +154,25 @@
     <t>chick-mince-meatballs-w4</t>
   </si>
   <si>
-    <t>Куриные тефтели в томатно-сметанном соусе</t>
+    <t>Куриные фрикадельки в соусе</t>
+  </si>
+  <si>
+    <t>chick-grill</t>
+  </si>
+  <si>
+    <t>филе</t>
+  </si>
+  <si>
+    <t>Филе куриное гриль</t>
+  </si>
+  <si>
+    <t>chicken-liver</t>
+  </si>
+  <si>
+    <t>печень</t>
+  </si>
+  <si>
+    <t>Куриная печень в сметане</t>
   </si>
   <si>
     <t>legs-w1</t>
@@ -169,12 +184,15 @@
     <t>1 кг</t>
   </si>
   <si>
-    <t>Ножки медово-чесночные / Ножки в паприке</t>
+    <t>Ножки медово-чесночные</t>
   </si>
   <si>
     <t>legs-w3</t>
   </si>
   <si>
+    <t>Ножки в паприке</t>
+  </si>
+  <si>
     <t>wings-w2</t>
   </si>
   <si>
@@ -193,10 +211,10 @@
     <t>бёдра</t>
   </si>
   <si>
-    <t>1,3 кг</t>
-  </si>
-  <si>
-    <t>Бёдра запечённые со сметаной и чесноком</t>
+    <t>800 г</t>
+  </si>
+  <si>
+    <t>Бёдра в грибном сметанном соусе</t>
   </si>
   <si>
     <t>trout-grill</t>
@@ -229,10 +247,13 @@
     <t>Минтай</t>
   </si>
   <si>
-    <t>Минтай запечённый с овощами и сыром</t>
-  </si>
-  <si>
-    <t>shrimp-rice-w1</t>
+    <t>750 г</t>
+  </si>
+  <si>
+    <t>Минтай с овощами и сыром</t>
+  </si>
+  <si>
+    <t>shrimp-pasta-w2</t>
   </si>
   <si>
     <t>Креветки</t>
@@ -241,10 +262,7 @@
     <t>целые</t>
   </si>
   <si>
-    <t>Золотой рис с креветками (Хайнань)</t>
-  </si>
-  <si>
-    <t>shrimp-pasta-w2</t>
+    <t>400 г</t>
   </si>
   <si>
     <t>Паста с креветками</t>
@@ -687,13 +705,13 @@
         <v>7</v>
       </c>
       <c r="C3" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="D3" t="s">
         <v>9</v>
       </c>
       <c r="E3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F3" t="s">
         <v>11</v>
@@ -701,13 +719,13 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B4" t="s">
         <v>7</v>
       </c>
       <c r="C4" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D4" t="s">
         <v>9</v>
@@ -727,13 +745,13 @@
         <v>7</v>
       </c>
       <c r="C5" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="D5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F5" t="s">
         <v>11</v>
@@ -741,19 +759,19 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B6" t="s">
         <v>7</v>
       </c>
       <c r="C6" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="D6" t="s">
-        <v>9</v>
+        <v>22</v>
       </c>
       <c r="E6" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="F6" t="s">
         <v>11</v>
@@ -761,19 +779,19 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="B7" t="s">
         <v>7</v>
       </c>
       <c r="C7" t="s">
+        <v>25</v>
+      </c>
+      <c r="D7" t="s">
         <v>22</v>
       </c>
-      <c r="D7" t="s">
-        <v>23</v>
-      </c>
       <c r="E7" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="F7" t="s">
         <v>11</v>
@@ -781,19 +799,19 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B8" t="s">
         <v>7</v>
       </c>
       <c r="C8" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D8" t="s">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="E8" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="F8" t="s">
         <v>11</v>
@@ -801,19 +819,19 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="B9" t="s">
         <v>7</v>
       </c>
       <c r="C9" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="D9" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="E9" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F9" t="s">
         <v>11</v>
@@ -821,190 +839,190 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B10" t="s">
-        <v>7</v>
+        <v>33</v>
       </c>
       <c r="C10" t="s">
-        <v>28</v>
+        <v>13</v>
       </c>
       <c r="D10" t="s">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="E10" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="F10" t="s">
-        <v>11</v>
+        <v>35</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>36</v>
+      </c>
+      <c r="B11" t="s">
         <v>33</v>
       </c>
-      <c r="B11" t="s">
-        <v>34</v>
-      </c>
       <c r="C11" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D11" t="s">
-        <v>9</v>
+        <v>37</v>
       </c>
       <c r="E11" t="s">
+        <v>38</v>
+      </c>
+      <c r="F11" t="s">
         <v>35</v>
-      </c>
-      <c r="F11" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B12" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C12" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="D12" t="s">
-        <v>38</v>
+        <v>9</v>
       </c>
       <c r="E12" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F12" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B13" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C13" t="s">
-        <v>8</v>
+        <v>42</v>
       </c>
       <c r="D13" t="s">
         <v>9</v>
       </c>
       <c r="E13" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="F13" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B14" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C14" t="s">
-        <v>43</v>
+        <v>25</v>
       </c>
       <c r="D14" t="s">
         <v>9</v>
       </c>
       <c r="E14" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F14" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B15" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C15" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="D15" t="s">
         <v>9</v>
       </c>
       <c r="E15" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F15" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B16" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C16" t="s">
-        <v>28</v>
+        <v>49</v>
       </c>
       <c r="D16" t="s">
-        <v>29</v>
+        <v>9</v>
       </c>
       <c r="E16" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="F16" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B17" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C17" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D17" t="s">
-        <v>51</v>
+        <v>9</v>
       </c>
       <c r="E17" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="F17" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B18" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C18" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="D18" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="E18" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="F18" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="B19" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C19" t="s">
         <v>55</v>
@@ -1013,50 +1031,50 @@
         <v>56</v>
       </c>
       <c r="E19" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F19" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B20" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C20" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D20" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="E20" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="F20" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B21" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="C21" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D21" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E21" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="F21" t="s">
-        <v>67</v>
+        <v>35</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
@@ -1064,79 +1082,79 @@
         <v>68</v>
       </c>
       <c r="B22" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="C22" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="D22" t="s">
-        <v>18</v>
+        <v>71</v>
       </c>
       <c r="E22" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="F22" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
+        <v>74</v>
+      </c>
+      <c r="B23" t="s">
+        <v>69</v>
+      </c>
+      <c r="C23" t="s">
         <v>70</v>
       </c>
-      <c r="B23" t="s">
-        <v>71</v>
-      </c>
-      <c r="C23" t="s">
-        <v>64</v>
-      </c>
       <c r="D23" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="E23" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="F23" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
+        <v>76</v>
+      </c>
+      <c r="B24" t="s">
+        <v>77</v>
+      </c>
+      <c r="C24" t="s">
+        <v>70</v>
+      </c>
+      <c r="D24" t="s">
+        <v>78</v>
+      </c>
+      <c r="E24" t="s">
+        <v>79</v>
+      </c>
+      <c r="F24" t="s">
         <v>73</v>
-      </c>
-      <c r="B24" t="s">
-        <v>74</v>
-      </c>
-      <c r="C24" t="s">
-        <v>75</v>
-      </c>
-      <c r="D24" t="s">
-        <v>23</v>
-      </c>
-      <c r="E24" t="s">
-        <v>76</v>
-      </c>
-      <c r="F24" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="B25" t="s">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="C25" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="D25" t="s">
-        <v>23</v>
+        <v>83</v>
       </c>
       <c r="E25" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="F25" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
     </row>
   </sheetData>

</xml_diff>